<commit_message>
fix: category filter, data mode toggle, model page month filter
</commit_message>
<xml_diff>
--- a/data/Tonor/Feb/Sp&Sd.xlsx
+++ b/data/Tonor/Feb/Sp&Sd.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\09-04-26\Sp-sd\AA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\buybox\data\Tonor\Feb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA286464-F86C-4F82-9B87-B635BC42F9BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{742BC802-0EAB-48A1-92FC-8934897B33EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C2EB3544-0B30-4B5A-9817-98DE85FBF6BC}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SB!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SD!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SP!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SP!$A$1:$I$1711</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">SP_SD_Combined!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10347" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10571" uniqueCount="82">
   <si>
     <t>Brand</t>
   </si>
@@ -284,6 +284,12 @@
   <si>
     <t>B07JMYG6LF</t>
   </si>
+  <si>
+    <t>Ton_Condenser_TC-777_SBV_KT</t>
+  </si>
+  <si>
+    <t>Ton_Dynamic_K1_SBV_KT</t>
+  </si>
 </sst>
 </file>
 
@@ -292,13 +298,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$₹-409]#,##0.00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -309,7 +321,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -317,16 +329,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -642,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51EF6D63-3663-4E20-A7FC-263D078FDDB8}">
-  <dimension ref="A1:I1655"/>
+  <dimension ref="A1:I1711"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.88671875" customWidth="1"/>
@@ -48643,7 +48673,1632 @@
         <v>9</v>
       </c>
     </row>
+    <row r="1656" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1656" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1656" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1656" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1656" s="1">
+        <v>2336</v>
+      </c>
+      <c r="E1656" s="1">
+        <v>7</v>
+      </c>
+      <c r="F1656" s="2">
+        <v>49.81</v>
+      </c>
+      <c r="G1656" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1656" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1656" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1657" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1657" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1657" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1657" s="1">
+        <v>5446</v>
+      </c>
+      <c r="E1657" s="1">
+        <v>7</v>
+      </c>
+      <c r="F1657" s="2">
+        <v>55.44</v>
+      </c>
+      <c r="G1657" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1657" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1657" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1658" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1658" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1658" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1658" s="1">
+        <v>3975</v>
+      </c>
+      <c r="E1658" s="1">
+        <v>6</v>
+      </c>
+      <c r="F1658" s="2">
+        <v>30.22</v>
+      </c>
+      <c r="G1658" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1658" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1658" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1659" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1659" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1659" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1659" s="1">
+        <v>587</v>
+      </c>
+      <c r="E1659" s="1">
+        <v>3</v>
+      </c>
+      <c r="F1659" s="2">
+        <v>18.86</v>
+      </c>
+      <c r="G1659" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1659" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1659" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1660" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1660" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1660" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1660" s="1">
+        <v>653</v>
+      </c>
+      <c r="E1660" s="1">
+        <v>4</v>
+      </c>
+      <c r="F1660" s="2">
+        <v>19.760000000000002</v>
+      </c>
+      <c r="G1660" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1660" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1660" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1661" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1661" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1661" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1661" s="1">
+        <v>705</v>
+      </c>
+      <c r="E1661" s="1">
+        <v>1</v>
+      </c>
+      <c r="F1661" s="2">
+        <v>5.34</v>
+      </c>
+      <c r="G1661" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1661" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1661" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1662" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1662" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1662" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1662" s="1">
+        <v>1070</v>
+      </c>
+      <c r="E1662" s="1">
+        <v>4</v>
+      </c>
+      <c r="F1662" s="2">
+        <v>37.21</v>
+      </c>
+      <c r="G1662" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1662" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1662" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1663" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1663" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1663" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1663" s="1">
+        <v>1782</v>
+      </c>
+      <c r="E1663" s="1">
+        <v>10</v>
+      </c>
+      <c r="F1663" s="2">
+        <v>108.97</v>
+      </c>
+      <c r="G1663" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1663" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1663" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1664" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1664" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1664" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1664" s="1">
+        <v>2010</v>
+      </c>
+      <c r="E1664" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1664" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1664" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1664" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1664" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1665" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1665" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1665" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1665" s="1">
+        <v>2589</v>
+      </c>
+      <c r="E1665" s="1">
+        <v>7</v>
+      </c>
+      <c r="F1665" s="2">
+        <v>81.88</v>
+      </c>
+      <c r="G1665" s="2">
+        <v>1905.93</v>
+      </c>
+      <c r="H1665" s="1">
+        <v>1</v>
+      </c>
+      <c r="I1665" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1666" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1666" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1666" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1666" s="1">
+        <v>519</v>
+      </c>
+      <c r="E1666" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1666" s="2">
+        <v>14.73</v>
+      </c>
+      <c r="G1666" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1666" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1666" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1667" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1667" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1667" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1667" s="1">
+        <v>3057</v>
+      </c>
+      <c r="E1667" s="1">
+        <v>4</v>
+      </c>
+      <c r="F1667" s="2">
+        <v>46.33</v>
+      </c>
+      <c r="G1667" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1667" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1667" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1668" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1668" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1668" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1668" s="1">
+        <v>722</v>
+      </c>
+      <c r="E1668" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1668" s="2">
+        <v>9.25</v>
+      </c>
+      <c r="G1668" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1668" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1668" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1669" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1669" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1669" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1669" s="1">
+        <v>586</v>
+      </c>
+      <c r="E1669" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1669" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1669" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1669" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1669" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1670" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1670" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1670" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1670" s="1">
+        <v>594</v>
+      </c>
+      <c r="E1670" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1670" s="2">
+        <v>8.92</v>
+      </c>
+      <c r="G1670" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1670" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1670" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1671" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1671" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1671" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1671" s="1">
+        <v>499</v>
+      </c>
+      <c r="E1671" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1671" s="2">
+        <v>16.64</v>
+      </c>
+      <c r="G1671" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1671" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1671" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1672" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1672" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1672" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1672" s="1">
+        <v>347</v>
+      </c>
+      <c r="E1672" s="1">
+        <v>1</v>
+      </c>
+      <c r="F1672" s="2">
+        <v>12.62</v>
+      </c>
+      <c r="G1672" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1672" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1672" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1673" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1673" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1673" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1673" s="1">
+        <v>496</v>
+      </c>
+      <c r="E1673" s="1">
+        <v>1</v>
+      </c>
+      <c r="F1673" s="2">
+        <v>6</v>
+      </c>
+      <c r="G1673" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1673" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1673" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1674" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1674" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1674" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1674" s="1">
+        <v>1961</v>
+      </c>
+      <c r="E1674" s="1">
+        <v>3</v>
+      </c>
+      <c r="F1674" s="2">
+        <v>20.38</v>
+      </c>
+      <c r="G1674" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1674" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1674" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1675" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1675" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1675" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1675" s="1">
+        <v>1274</v>
+      </c>
+      <c r="E1675" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1675" s="2">
+        <v>13.66</v>
+      </c>
+      <c r="G1675" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1675" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1675" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1676" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1676" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1676" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1676" s="1">
+        <v>312</v>
+      </c>
+      <c r="E1676" s="1">
+        <v>3</v>
+      </c>
+      <c r="F1676" s="2">
+        <v>13.87</v>
+      </c>
+      <c r="G1676" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1676" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1676" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1677" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1677" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1677" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1677" s="1">
+        <v>888</v>
+      </c>
+      <c r="E1677" s="1">
+        <v>11</v>
+      </c>
+      <c r="F1677" s="2">
+        <v>126.08</v>
+      </c>
+      <c r="G1677" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1677" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1677" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1678" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1678" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1678" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1678" s="1">
+        <v>594</v>
+      </c>
+      <c r="E1678" s="1">
+        <v>15</v>
+      </c>
+      <c r="F1678" s="2">
+        <v>177.73</v>
+      </c>
+      <c r="G1678" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1678" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1678" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1679" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1679" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1679" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1679" s="1">
+        <v>746</v>
+      </c>
+      <c r="E1679" s="1">
+        <v>11</v>
+      </c>
+      <c r="F1679" s="2">
+        <v>121.23</v>
+      </c>
+      <c r="G1679" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1679" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1679" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1680" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1680" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1680" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1680" s="1">
+        <v>659</v>
+      </c>
+      <c r="E1680" s="1">
+        <v>14</v>
+      </c>
+      <c r="F1680" s="2">
+        <v>218.51</v>
+      </c>
+      <c r="G1680" s="2">
+        <v>1524.58</v>
+      </c>
+      <c r="H1680" s="1">
+        <v>2</v>
+      </c>
+      <c r="I1680" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1681" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1681" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1681" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1681" s="1">
+        <v>437</v>
+      </c>
+      <c r="E1681" s="1">
+        <v>6</v>
+      </c>
+      <c r="F1681" s="2">
+        <v>78.62</v>
+      </c>
+      <c r="G1681" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1681" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1681" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1682" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1682" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1682" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1682" s="1">
+        <v>472</v>
+      </c>
+      <c r="E1682" s="1">
+        <v>12</v>
+      </c>
+      <c r="F1682" s="2">
+        <v>122.13</v>
+      </c>
+      <c r="G1682" s="2">
+        <v>1524.58</v>
+      </c>
+      <c r="H1682" s="1">
+        <v>1</v>
+      </c>
+      <c r="I1682" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1683" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1683" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1683" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1683" s="1">
+        <v>536</v>
+      </c>
+      <c r="E1683" s="1">
+        <v>8</v>
+      </c>
+      <c r="F1683" s="2">
+        <v>63.95</v>
+      </c>
+      <c r="G1683" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1683" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1683" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1684" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1684" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1684" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1684" s="1">
+        <v>703</v>
+      </c>
+      <c r="E1684" s="1">
+        <v>11</v>
+      </c>
+      <c r="F1684" s="2">
+        <v>100.03</v>
+      </c>
+      <c r="G1684" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1684" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1684" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1685" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1685" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1685" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1685" s="1">
+        <v>615</v>
+      </c>
+      <c r="E1685" s="1">
+        <v>9</v>
+      </c>
+      <c r="F1685" s="2">
+        <v>84.8</v>
+      </c>
+      <c r="G1685" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1685" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1685" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1686" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1686" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1686" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1686" s="1">
+        <v>716</v>
+      </c>
+      <c r="E1686" s="1">
+        <v>14</v>
+      </c>
+      <c r="F1686" s="2">
+        <v>111.73</v>
+      </c>
+      <c r="G1686" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1686" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1686" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1687" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1687" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1687" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1687" s="1">
+        <v>610</v>
+      </c>
+      <c r="E1687" s="1">
+        <v>12</v>
+      </c>
+      <c r="F1687" s="2">
+        <v>98</v>
+      </c>
+      <c r="G1687" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1687" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1687" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1688" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1688" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1688" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1688" s="1">
+        <v>751</v>
+      </c>
+      <c r="E1688" s="1">
+        <v>15</v>
+      </c>
+      <c r="F1688" s="2">
+        <v>122.62</v>
+      </c>
+      <c r="G1688" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1688" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1688" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1689" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1689" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1689" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1689" s="1">
+        <v>416</v>
+      </c>
+      <c r="E1689" s="1">
+        <v>4</v>
+      </c>
+      <c r="F1689" s="2">
+        <v>36.090000000000003</v>
+      </c>
+      <c r="G1689" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1689" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1689" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1690" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1690" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1690" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1690" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1690" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1690" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1690" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1690" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1690" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1691" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1691" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1691" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1691" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1691" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1691" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1691" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1691" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1691" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1692" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1692" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1692" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1692" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1692" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1692" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1692" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1692" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1692" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1693" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1693" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1693" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1693" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1693" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1693" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1693" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1693" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1693" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1694" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1694" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1694" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1694" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1694" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1694" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1694" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1694" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1694" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1695" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1695" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1695" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1695" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1695" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1695" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1695" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1695" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1695" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1696" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1696" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1696" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1696" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1696" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1696" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1696" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1696" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1696" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1697" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1697" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1697" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1697" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1697" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1697" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1697" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1697" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1697" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1698" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1698" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1698" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1698" s="1">
+        <v>426</v>
+      </c>
+      <c r="E1698" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1698" s="2">
+        <v>25.88</v>
+      </c>
+      <c r="G1698" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1698" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1698" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1699" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1699" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1699" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1699" s="1">
+        <v>1136</v>
+      </c>
+      <c r="E1699" s="1">
+        <v>2</v>
+      </c>
+      <c r="F1699" s="2">
+        <v>8</v>
+      </c>
+      <c r="G1699" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1699" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1699" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1700" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1700" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1700" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1700" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1700" s="1">
+        <v>191</v>
+      </c>
+      <c r="E1700" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1700" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1700" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1700" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1700" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1701" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1701" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1701" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1701" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1701" s="1">
+        <v>211</v>
+      </c>
+      <c r="E1701" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1701" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1701" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1701" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1701" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1702" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1702" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1702" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1702" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1702" s="1">
+        <v>239</v>
+      </c>
+      <c r="E1702" s="1">
+        <v>1</v>
+      </c>
+      <c r="F1702" s="2">
+        <v>4.78</v>
+      </c>
+      <c r="G1702" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1702" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1702" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1703" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1703" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1703" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1703" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1703" s="1">
+        <v>317</v>
+      </c>
+      <c r="E1703" s="1">
+        <v>3</v>
+      </c>
+      <c r="F1703" s="2">
+        <v>34.81</v>
+      </c>
+      <c r="G1703" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1703" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1703" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1704" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1704" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1704" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1704" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1704" s="1">
+        <v>3030</v>
+      </c>
+      <c r="E1704" s="1">
+        <v>5</v>
+      </c>
+      <c r="F1704" s="2">
+        <v>76.05</v>
+      </c>
+      <c r="G1704" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1704" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1704" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1705" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1705" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1705" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1705" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1705" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1705" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1705" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1705" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1705" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1705" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1706" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1706" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1706" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1706" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1706" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1706" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1706" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1706" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1706" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1706" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1707" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1707" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1707" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1707" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1707" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1707" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1707" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1707" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1707" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1707" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1708" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1708" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1708" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1708" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1708" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1708" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1708" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1708" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1708" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1708" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1709" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1709" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1709" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1709" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1709" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1709" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1709" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1709" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1709" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1709" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1710" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1710" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1710" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1710" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1710" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1710" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1710" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1710" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1710" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1710" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1711" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1711" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1711" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1711" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1711" s="1">
+        <v>0</v>
+      </c>
+      <c r="F1711" s="2">
+        <v>0</v>
+      </c>
+      <c r="G1711" s="2">
+        <v>0</v>
+      </c>
+      <c r="H1711" s="1">
+        <v>0</v>
+      </c>
+      <c r="I1711" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:I1711" xr:uid="{51EF6D63-3663-4E20-A7FC-263D078FDDB8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>